<commit_message>
created final energy mapping and cleaned scripts for readability
</commit_message>
<xml_diff>
--- a/gcam/output/SSP2/iamc_template_gcam_other.xlsx
+++ b/gcam/output/SSP2/iamc_template_gcam_other.xlsx
@@ -684,70 +684,70 @@
         <v>66</v>
       </c>
       <c r="F2">
-        <v>98409</v>
+        <v>98.40900000000001</v>
       </c>
       <c r="G2">
-        <v>151062</v>
+        <v>151.062</v>
       </c>
       <c r="H2">
-        <v>230484</v>
+        <v>230.484</v>
       </c>
       <c r="I2">
-        <v>266642</v>
+        <v>266.642</v>
       </c>
       <c r="J2">
-        <v>304443</v>
+        <v>304.443</v>
       </c>
       <c r="K2">
-        <v>355355</v>
+        <v>355.355</v>
       </c>
       <c r="L2">
-        <v>391100</v>
+        <v>391.1</v>
       </c>
       <c r="M2">
-        <v>438024</v>
+        <v>438.024</v>
       </c>
       <c r="N2">
-        <v>485635</v>
+        <v>485.635</v>
       </c>
       <c r="O2">
-        <v>532794</v>
+        <v>532.794</v>
       </c>
       <c r="P2">
-        <v>578897</v>
+        <v>578.897</v>
       </c>
       <c r="Q2">
-        <v>623428</v>
+        <v>623.428</v>
       </c>
       <c r="R2">
-        <v>665230</v>
+        <v>665.23</v>
       </c>
       <c r="S2">
-        <v>704017</v>
+        <v>704.0170000000001</v>
       </c>
       <c r="T2">
-        <v>738606</v>
+        <v>738.606</v>
       </c>
       <c r="U2">
-        <v>768862</v>
+        <v>768.862</v>
       </c>
       <c r="V2">
-        <v>793943</v>
+        <v>793.943</v>
       </c>
       <c r="W2">
-        <v>814205</v>
+        <v>814.205</v>
       </c>
       <c r="X2">
-        <v>830143</v>
+        <v>830.143</v>
       </c>
       <c r="Y2">
-        <v>842266</v>
+        <v>842.266</v>
       </c>
       <c r="Z2">
-        <v>850642</v>
+        <v>850.6420000000001</v>
       </c>
       <c r="AA2">
-        <v>855535</v>
+        <v>855.535</v>
       </c>
     </row>
     <row r="3" spans="1:27">
@@ -767,70 +767,70 @@
         <v>66</v>
       </c>
       <c r="F3">
-        <v>79953</v>
+        <v>79.953</v>
       </c>
       <c r="G3">
-        <v>120159</v>
+        <v>120.159</v>
       </c>
       <c r="H3">
-        <v>159029</v>
+        <v>159.029</v>
       </c>
       <c r="I3">
-        <v>173374</v>
+        <v>173.374</v>
       </c>
       <c r="J3">
-        <v>190189</v>
+        <v>190.189</v>
       </c>
       <c r="K3">
-        <v>210081</v>
+        <v>210.081</v>
       </c>
       <c r="L3">
-        <v>222993</v>
+        <v>222.993</v>
       </c>
       <c r="M3">
-        <v>238346</v>
+        <v>238.346</v>
       </c>
       <c r="N3">
-        <v>253020</v>
+        <v>253.02</v>
       </c>
       <c r="O3">
-        <v>267277</v>
+        <v>267.277</v>
       </c>
       <c r="P3">
-        <v>280708</v>
+        <v>280.708</v>
       </c>
       <c r="Q3">
-        <v>292805</v>
+        <v>292.805</v>
       </c>
       <c r="R3">
-        <v>303162</v>
+        <v>303.162</v>
       </c>
       <c r="S3">
-        <v>311731</v>
+        <v>311.731</v>
       </c>
       <c r="T3">
-        <v>318383</v>
+        <v>318.383</v>
       </c>
       <c r="U3">
-        <v>323405</v>
+        <v>323.405</v>
       </c>
       <c r="V3">
-        <v>327298</v>
+        <v>327.298</v>
       </c>
       <c r="W3">
-        <v>330277</v>
+        <v>330.277</v>
       </c>
       <c r="X3">
-        <v>332354</v>
+        <v>332.354</v>
       </c>
       <c r="Y3">
-        <v>333628</v>
+        <v>333.628</v>
       </c>
       <c r="Z3">
-        <v>333848</v>
+        <v>333.848</v>
       </c>
       <c r="AA3">
-        <v>332951</v>
+        <v>332.951</v>
       </c>
     </row>
     <row r="4" spans="1:27">
@@ -850,70 +850,70 @@
         <v>66</v>
       </c>
       <c r="F4">
-        <v>52620</v>
+        <v>52.62</v>
       </c>
       <c r="G4">
-        <v>84042</v>
+        <v>84.042</v>
       </c>
       <c r="H4">
-        <v>122552</v>
+        <v>122.552</v>
       </c>
       <c r="I4">
-        <v>140212</v>
+        <v>140.212</v>
       </c>
       <c r="J4">
-        <v>162696</v>
+        <v>162.696</v>
       </c>
       <c r="K4">
-        <v>194118</v>
+        <v>194.118</v>
       </c>
       <c r="L4">
-        <v>215688</v>
+        <v>215.688</v>
       </c>
       <c r="M4">
-        <v>244055</v>
+        <v>244.055</v>
       </c>
       <c r="N4">
-        <v>273381</v>
+        <v>273.381</v>
       </c>
       <c r="O4">
-        <v>303131</v>
+        <v>303.131</v>
       </c>
       <c r="P4">
-        <v>332760</v>
+        <v>332.76</v>
       </c>
       <c r="Q4">
-        <v>361618</v>
+        <v>361.618</v>
       </c>
       <c r="R4">
-        <v>388966</v>
+        <v>388.966</v>
       </c>
       <c r="S4">
-        <v>414621</v>
+        <v>414.621</v>
       </c>
       <c r="T4">
-        <v>438016</v>
+        <v>438.016</v>
       </c>
       <c r="U4">
-        <v>458830</v>
+        <v>458.83</v>
       </c>
       <c r="V4">
-        <v>476989</v>
+        <v>476.989</v>
       </c>
       <c r="W4">
-        <v>491948</v>
+        <v>491.948</v>
       </c>
       <c r="X4">
-        <v>503434</v>
+        <v>503.434</v>
       </c>
       <c r="Y4">
-        <v>511665</v>
+        <v>511.665</v>
       </c>
       <c r="Z4">
-        <v>517324</v>
+        <v>517.324</v>
       </c>
       <c r="AA4">
-        <v>520771</v>
+        <v>520.771</v>
       </c>
     </row>
     <row r="5" spans="1:27">
@@ -933,70 +933,70 @@
         <v>66</v>
       </c>
       <c r="F5">
-        <v>160687</v>
+        <v>160.687</v>
       </c>
       <c r="G5">
-        <v>242847</v>
+        <v>242.847</v>
       </c>
       <c r="H5">
-        <v>366537</v>
+        <v>366.537</v>
       </c>
       <c r="I5">
-        <v>422911</v>
+        <v>422.911</v>
       </c>
       <c r="J5">
-        <v>487548</v>
+        <v>487.548</v>
       </c>
       <c r="K5">
-        <v>574303</v>
+        <v>574.303</v>
       </c>
       <c r="L5">
-        <v>637591</v>
+        <v>637.591</v>
       </c>
       <c r="M5">
-        <v>723488</v>
+        <v>723.4880000000001</v>
       </c>
       <c r="N5">
-        <v>815076</v>
+        <v>815.076</v>
       </c>
       <c r="O5">
-        <v>911381</v>
+        <v>911.381</v>
       </c>
       <c r="P5">
-        <v>1010580</v>
+        <v>1010.58</v>
       </c>
       <c r="Q5">
-        <v>1110720</v>
+        <v>1110.72</v>
       </c>
       <c r="R5">
-        <v>1209160</v>
+        <v>1209.16</v>
       </c>
       <c r="S5">
-        <v>1304450</v>
+        <v>1304.45</v>
       </c>
       <c r="T5">
-        <v>1395550</v>
+        <v>1395.55</v>
       </c>
       <c r="U5">
-        <v>1481360</v>
+        <v>1481.36</v>
       </c>
       <c r="V5">
-        <v>1560780</v>
+        <v>1560.78</v>
       </c>
       <c r="W5">
-        <v>1632350</v>
+        <v>1632.35</v>
       </c>
       <c r="X5">
-        <v>1695070</v>
+        <v>1695.07</v>
       </c>
       <c r="Y5">
-        <v>1748160</v>
+        <v>1748.16</v>
       </c>
       <c r="Z5">
-        <v>1790820</v>
+        <v>1790.82</v>
       </c>
       <c r="AA5">
-        <v>1823070</v>
+        <v>1823.07</v>
       </c>
     </row>
     <row r="6" spans="1:27">
@@ -1016,70 +1016,70 @@
         <v>66</v>
       </c>
       <c r="F6">
-        <v>25876</v>
+        <v>25.876</v>
       </c>
       <c r="G6">
-        <v>32638</v>
+        <v>32.638</v>
       </c>
       <c r="H6">
-        <v>39071</v>
+        <v>39.071</v>
       </c>
       <c r="I6">
-        <v>41100</v>
+        <v>41.1</v>
       </c>
       <c r="J6">
-        <v>43257</v>
+        <v>43.257</v>
       </c>
       <c r="K6">
-        <v>45277</v>
+        <v>45.277</v>
       </c>
       <c r="L6">
-        <v>46190</v>
+        <v>46.19</v>
       </c>
       <c r="M6">
-        <v>47373</v>
+        <v>47.373</v>
       </c>
       <c r="N6">
-        <v>48471</v>
+        <v>48.471</v>
       </c>
       <c r="O6">
-        <v>49452</v>
+        <v>49.452</v>
       </c>
       <c r="P6">
-        <v>50276</v>
+        <v>50.276</v>
       </c>
       <c r="Q6">
-        <v>50923</v>
+        <v>50.923</v>
       </c>
       <c r="R6">
-        <v>51384</v>
+        <v>51.384</v>
       </c>
       <c r="S6">
-        <v>51617</v>
+        <v>51.617</v>
       </c>
       <c r="T6">
-        <v>51654</v>
+        <v>51.654</v>
       </c>
       <c r="U6">
-        <v>51525</v>
+        <v>51.525</v>
       </c>
       <c r="V6">
-        <v>51242</v>
+        <v>51.242</v>
       </c>
       <c r="W6">
-        <v>50814</v>
+        <v>50.814</v>
       </c>
       <c r="X6">
-        <v>50249</v>
+        <v>50.249</v>
       </c>
       <c r="Y6">
-        <v>49567</v>
+        <v>49.567</v>
       </c>
       <c r="Z6">
-        <v>48790</v>
+        <v>48.79</v>
       </c>
       <c r="AA6">
-        <v>47947</v>
+        <v>47.947</v>
       </c>
     </row>
     <row r="7" spans="1:27">
@@ -1099,70 +1099,70 @@
         <v>66</v>
       </c>
       <c r="F7">
-        <v>16982</v>
+        <v>16.982</v>
       </c>
       <c r="G7">
-        <v>20445</v>
+        <v>20.445</v>
       </c>
       <c r="H7">
-        <v>24305</v>
+        <v>24.305</v>
       </c>
       <c r="I7">
-        <v>26366</v>
+        <v>26.366</v>
       </c>
       <c r="J7">
-        <v>28411</v>
+        <v>28.411</v>
       </c>
       <c r="K7">
-        <v>31051</v>
+        <v>31.051</v>
       </c>
       <c r="L7">
-        <v>31999</v>
+        <v>31.999</v>
       </c>
       <c r="M7">
-        <v>33135</v>
+        <v>33.135</v>
       </c>
       <c r="N7">
-        <v>34189</v>
+        <v>34.189</v>
       </c>
       <c r="O7">
-        <v>35181</v>
+        <v>35.181</v>
       </c>
       <c r="P7">
-        <v>36154</v>
+        <v>36.154</v>
       </c>
       <c r="Q7">
-        <v>37135</v>
+        <v>37.135</v>
       </c>
       <c r="R7">
-        <v>38039</v>
+        <v>38.039</v>
       </c>
       <c r="S7">
-        <v>38872</v>
+        <v>38.872</v>
       </c>
       <c r="T7">
-        <v>39592</v>
+        <v>39.592</v>
       </c>
       <c r="U7">
-        <v>40214</v>
+        <v>40.214</v>
       </c>
       <c r="V7">
-        <v>40732</v>
+        <v>40.732</v>
       </c>
       <c r="W7">
-        <v>41128</v>
+        <v>41.128</v>
       </c>
       <c r="X7">
-        <v>41369</v>
+        <v>41.369</v>
       </c>
       <c r="Y7">
-        <v>41451</v>
+        <v>41.451</v>
       </c>
       <c r="Z7">
-        <v>41406</v>
+        <v>41.406</v>
       </c>
       <c r="AA7">
-        <v>41268</v>
+        <v>41.268</v>
       </c>
     </row>
     <row r="8" spans="1:27">
@@ -1182,70 +1182,70 @@
         <v>66</v>
       </c>
       <c r="F8">
-        <v>108701</v>
+        <v>108.701</v>
       </c>
       <c r="G8">
-        <v>150706</v>
+        <v>150.706</v>
       </c>
       <c r="H8">
-        <v>186797</v>
+        <v>186.797</v>
       </c>
       <c r="I8">
-        <v>196353</v>
+        <v>196.353</v>
       </c>
       <c r="J8">
-        <v>205188</v>
+        <v>205.188</v>
       </c>
       <c r="K8">
-        <v>214326</v>
+        <v>214.326</v>
       </c>
       <c r="L8">
-        <v>218338</v>
+        <v>218.338</v>
       </c>
       <c r="M8">
-        <v>223013</v>
+        <v>223.013</v>
       </c>
       <c r="N8">
-        <v>226408</v>
+        <v>226.408</v>
       </c>
       <c r="O8">
-        <v>228456</v>
+        <v>228.456</v>
       </c>
       <c r="P8">
-        <v>229197</v>
+        <v>229.197</v>
       </c>
       <c r="Q8">
-        <v>228626</v>
+        <v>228.626</v>
       </c>
       <c r="R8">
-        <v>226961</v>
+        <v>226.961</v>
       </c>
       <c r="S8">
-        <v>224325</v>
+        <v>224.325</v>
       </c>
       <c r="T8">
-        <v>220772</v>
+        <v>220.772</v>
       </c>
       <c r="U8">
-        <v>216432</v>
+        <v>216.432</v>
       </c>
       <c r="V8">
-        <v>211422</v>
+        <v>211.422</v>
       </c>
       <c r="W8">
-        <v>205847</v>
+        <v>205.847</v>
       </c>
       <c r="X8">
-        <v>200021</v>
+        <v>200.021</v>
       </c>
       <c r="Y8">
-        <v>194117</v>
+        <v>194.117</v>
       </c>
       <c r="Z8">
-        <v>188295</v>
+        <v>188.295</v>
       </c>
       <c r="AA8">
-        <v>182660</v>
+        <v>182.66</v>
       </c>
     </row>
     <row r="9" spans="1:27">
@@ -1265,70 +1265,70 @@
         <v>66</v>
       </c>
       <c r="F9">
-        <v>23136</v>
+        <v>23.136</v>
       </c>
       <c r="G9">
-        <v>27657</v>
+        <v>27.657</v>
       </c>
       <c r="H9">
-        <v>32216</v>
+        <v>32.216</v>
       </c>
       <c r="I9">
-        <v>33963</v>
+        <v>33.963</v>
       </c>
       <c r="J9">
-        <v>35732</v>
+        <v>35.732</v>
       </c>
       <c r="K9">
-        <v>38155</v>
+        <v>38.155</v>
       </c>
       <c r="L9">
-        <v>38867</v>
+        <v>38.867</v>
       </c>
       <c r="M9">
-        <v>39671</v>
+        <v>39.671</v>
       </c>
       <c r="N9">
-        <v>40419</v>
+        <v>40.419</v>
       </c>
       <c r="O9">
-        <v>41100</v>
+        <v>41.1</v>
       </c>
       <c r="P9">
-        <v>41745</v>
+        <v>41.745</v>
       </c>
       <c r="Q9">
-        <v>42415</v>
+        <v>42.415</v>
       </c>
       <c r="R9">
-        <v>42986</v>
+        <v>42.986</v>
       </c>
       <c r="S9">
-        <v>43524</v>
+        <v>43.524</v>
       </c>
       <c r="T9">
-        <v>44019</v>
+        <v>44.019</v>
       </c>
       <c r="U9">
-        <v>44480</v>
+        <v>44.48</v>
       </c>
       <c r="V9">
-        <v>44859</v>
+        <v>44.859</v>
       </c>
       <c r="W9">
-        <v>45106</v>
+        <v>45.106</v>
       </c>
       <c r="X9">
-        <v>45187</v>
+        <v>45.187</v>
       </c>
       <c r="Y9">
-        <v>45099</v>
+        <v>45.099</v>
       </c>
       <c r="Z9">
-        <v>44874</v>
+        <v>44.874</v>
       </c>
       <c r="AA9">
-        <v>44547</v>
+        <v>44.547</v>
       </c>
     </row>
     <row r="10" spans="1:27">
@@ -1348,70 +1348,70 @@
         <v>66</v>
       </c>
       <c r="F10">
-        <v>45072</v>
+        <v>45.072</v>
       </c>
       <c r="G10">
-        <v>60084</v>
+        <v>60.084</v>
       </c>
       <c r="H10">
-        <v>76123</v>
+        <v>76.123</v>
       </c>
       <c r="I10">
-        <v>81118</v>
+        <v>81.11799999999999</v>
       </c>
       <c r="J10">
-        <v>86189</v>
+        <v>86.18899999999999</v>
       </c>
       <c r="K10">
-        <v>91771</v>
+        <v>91.771</v>
       </c>
       <c r="L10">
-        <v>95375</v>
+        <v>95.375</v>
       </c>
       <c r="M10">
-        <v>99761</v>
+        <v>99.761</v>
       </c>
       <c r="N10">
-        <v>103585</v>
+        <v>103.585</v>
       </c>
       <c r="O10">
-        <v>106763</v>
+        <v>106.763</v>
       </c>
       <c r="P10">
-        <v>109254</v>
+        <v>109.254</v>
       </c>
       <c r="Q10">
-        <v>111080</v>
+        <v>111.08</v>
       </c>
       <c r="R10">
-        <v>112270</v>
+        <v>112.27</v>
       </c>
       <c r="S10">
-        <v>112900</v>
+        <v>112.9</v>
       </c>
       <c r="T10">
-        <v>113102</v>
+        <v>113.102</v>
       </c>
       <c r="U10">
-        <v>112901</v>
+        <v>112.901</v>
       </c>
       <c r="V10">
-        <v>112318</v>
+        <v>112.318</v>
       </c>
       <c r="W10">
-        <v>111367</v>
+        <v>111.367</v>
       </c>
       <c r="X10">
-        <v>110109</v>
+        <v>110.109</v>
       </c>
       <c r="Y10">
-        <v>108612</v>
+        <v>108.612</v>
       </c>
       <c r="Z10">
-        <v>106947</v>
+        <v>106.947</v>
       </c>
       <c r="AA10">
-        <v>105200</v>
+        <v>105.2</v>
       </c>
     </row>
     <row r="11" spans="1:27">
@@ -1431,70 +1431,70 @@
         <v>66</v>
       </c>
       <c r="F11">
-        <v>51627</v>
+        <v>51.627</v>
       </c>
       <c r="G11">
-        <v>69516</v>
+        <v>69.51600000000001</v>
       </c>
       <c r="H11">
-        <v>77462</v>
+        <v>77.462</v>
       </c>
       <c r="I11">
-        <v>82338</v>
+        <v>82.33799999999999</v>
       </c>
       <c r="J11">
-        <v>88469</v>
+        <v>88.46899999999999</v>
       </c>
       <c r="K11">
-        <v>96107</v>
+        <v>96.107</v>
       </c>
       <c r="L11">
-        <v>100959</v>
+        <v>100.959</v>
       </c>
       <c r="M11">
-        <v>106386</v>
+        <v>106.386</v>
       </c>
       <c r="N11">
-        <v>111330</v>
+        <v>111.33</v>
       </c>
       <c r="O11">
-        <v>116062</v>
+        <v>116.062</v>
       </c>
       <c r="P11">
-        <v>120507</v>
+        <v>120.507</v>
       </c>
       <c r="Q11">
-        <v>124395</v>
+        <v>124.395</v>
       </c>
       <c r="R11">
-        <v>127451</v>
+        <v>127.451</v>
       </c>
       <c r="S11">
-        <v>129638</v>
+        <v>129.638</v>
       </c>
       <c r="T11">
-        <v>131189</v>
+        <v>131.189</v>
       </c>
       <c r="U11">
-        <v>132325</v>
+        <v>132.325</v>
       </c>
       <c r="V11">
-        <v>133117</v>
+        <v>133.117</v>
       </c>
       <c r="W11">
-        <v>133580</v>
+        <v>133.58</v>
       </c>
       <c r="X11">
-        <v>133768</v>
+        <v>133.768</v>
       </c>
       <c r="Y11">
-        <v>133722</v>
+        <v>133.722</v>
       </c>
       <c r="Z11">
-        <v>133474</v>
+        <v>133.474</v>
       </c>
       <c r="AA11">
-        <v>132935</v>
+        <v>132.935</v>
       </c>
     </row>
     <row r="12" spans="1:27">
@@ -1514,70 +1514,70 @@
         <v>66</v>
       </c>
       <c r="F12">
-        <v>919823</v>
+        <v>919.823</v>
       </c>
       <c r="G12">
-        <v>1159890</v>
+        <v>1159.89</v>
       </c>
       <c r="H12">
-        <v>1312310</v>
+        <v>1312.31</v>
       </c>
       <c r="I12">
-        <v>1355880</v>
+        <v>1355.88</v>
       </c>
       <c r="J12">
-        <v>1401730</v>
+        <v>1401.73</v>
       </c>
       <c r="K12">
-        <v>1434080</v>
+        <v>1434.08</v>
       </c>
       <c r="L12">
-        <v>1436020</v>
+        <v>1436.02</v>
       </c>
       <c r="M12">
-        <v>1425960</v>
+        <v>1425.96</v>
       </c>
       <c r="N12">
-        <v>1408520</v>
+        <v>1408.52</v>
       </c>
       <c r="O12">
-        <v>1385330</v>
+        <v>1385.33</v>
       </c>
       <c r="P12">
-        <v>1354900</v>
+        <v>1354.9</v>
       </c>
       <c r="Q12">
-        <v>1315550</v>
+        <v>1315.55</v>
       </c>
       <c r="R12">
-        <v>1267040</v>
+        <v>1267.04</v>
       </c>
       <c r="S12">
-        <v>1212540</v>
+        <v>1212.54</v>
       </c>
       <c r="T12">
-        <v>1155930</v>
+        <v>1155.93</v>
       </c>
       <c r="U12">
-        <v>1100670</v>
+        <v>1100.67</v>
       </c>
       <c r="V12">
-        <v>1047540</v>
+        <v>1047.54</v>
       </c>
       <c r="W12">
-        <v>995274</v>
+        <v>995.274</v>
       </c>
       <c r="X12">
-        <v>944011</v>
+        <v>944.011</v>
       </c>
       <c r="Y12">
-        <v>895579</v>
+        <v>895.579</v>
       </c>
       <c r="Z12">
-        <v>850710</v>
+        <v>850.71</v>
       </c>
       <c r="AA12">
-        <v>807888</v>
+        <v>807.888</v>
       </c>
     </row>
     <row r="13" spans="1:27">
@@ -1597,70 +1597,70 @@
         <v>66</v>
       </c>
       <c r="F13">
-        <v>23404</v>
+        <v>23.404</v>
       </c>
       <c r="G13">
-        <v>32601</v>
+        <v>32.601</v>
       </c>
       <c r="H13">
-        <v>42221</v>
+        <v>42.221</v>
       </c>
       <c r="I13">
-        <v>44816</v>
+        <v>44.816</v>
       </c>
       <c r="J13">
-        <v>47120</v>
+        <v>47.12</v>
       </c>
       <c r="K13">
-        <v>51517</v>
+        <v>51.517</v>
       </c>
       <c r="L13">
-        <v>52973</v>
+        <v>52.973</v>
       </c>
       <c r="M13">
-        <v>54767</v>
+        <v>54.767</v>
       </c>
       <c r="N13">
-        <v>56185</v>
+        <v>56.185</v>
       </c>
       <c r="O13">
-        <v>57224</v>
+        <v>57.224</v>
       </c>
       <c r="P13">
-        <v>57879</v>
+        <v>57.879</v>
       </c>
       <c r="Q13">
-        <v>58202</v>
+        <v>58.202</v>
       </c>
       <c r="R13">
-        <v>58246</v>
+        <v>58.246</v>
       </c>
       <c r="S13">
-        <v>58043</v>
+        <v>58.043</v>
       </c>
       <c r="T13">
-        <v>57622</v>
+        <v>57.622</v>
       </c>
       <c r="U13">
-        <v>56990</v>
+        <v>56.99</v>
       </c>
       <c r="V13">
-        <v>56160</v>
+        <v>56.16</v>
       </c>
       <c r="W13">
-        <v>55110</v>
+        <v>55.11</v>
       </c>
       <c r="X13">
-        <v>53912</v>
+        <v>53.912</v>
       </c>
       <c r="Y13">
-        <v>52638</v>
+        <v>52.638</v>
       </c>
       <c r="Z13">
-        <v>51356</v>
+        <v>51.356</v>
       </c>
       <c r="AA13">
-        <v>50132</v>
+        <v>50.132</v>
       </c>
     </row>
     <row r="14" spans="1:27">
@@ -1680,70 +1680,70 @@
         <v>66</v>
       </c>
       <c r="F14">
-        <v>99278</v>
+        <v>99.27800000000001</v>
       </c>
       <c r="G14">
-        <v>106793</v>
+        <v>106.793</v>
       </c>
       <c r="H14">
-        <v>103627</v>
+        <v>103.627</v>
       </c>
       <c r="I14">
-        <v>102551</v>
+        <v>102.551</v>
       </c>
       <c r="J14">
-        <v>101556</v>
+        <v>101.556</v>
       </c>
       <c r="K14">
-        <v>100070</v>
+        <v>100.07</v>
       </c>
       <c r="L14">
-        <v>99797</v>
+        <v>99.797</v>
       </c>
       <c r="M14">
-        <v>97571</v>
+        <v>97.571</v>
       </c>
       <c r="N14">
-        <v>95253</v>
+        <v>95.253</v>
       </c>
       <c r="O14">
-        <v>93009</v>
+        <v>93.009</v>
       </c>
       <c r="P14">
-        <v>90896</v>
+        <v>90.896</v>
       </c>
       <c r="Q14">
-        <v>88951</v>
+        <v>88.95099999999999</v>
       </c>
       <c r="R14">
-        <v>87014</v>
+        <v>87.014</v>
       </c>
       <c r="S14">
-        <v>85002</v>
+        <v>85.002</v>
       </c>
       <c r="T14">
-        <v>82866</v>
+        <v>82.866</v>
       </c>
       <c r="U14">
-        <v>80650</v>
+        <v>80.65000000000001</v>
       </c>
       <c r="V14">
-        <v>78463</v>
+        <v>78.46299999999999</v>
       </c>
       <c r="W14">
-        <v>76413</v>
+        <v>76.413</v>
       </c>
       <c r="X14">
-        <v>74562</v>
+        <v>74.562</v>
       </c>
       <c r="Y14">
-        <v>72919</v>
+        <v>72.919</v>
       </c>
       <c r="Z14">
-        <v>71450</v>
+        <v>71.45</v>
       </c>
       <c r="AA14">
-        <v>70064</v>
+        <v>70.06399999999999</v>
       </c>
     </row>
     <row r="15" spans="1:27">
@@ -1763,70 +1763,70 @@
         <v>66</v>
       </c>
       <c r="F15">
-        <v>349021</v>
+        <v>349.021</v>
       </c>
       <c r="G15">
-        <v>364582</v>
+        <v>364.582</v>
       </c>
       <c r="H15">
-        <v>385538</v>
+        <v>385.538</v>
       </c>
       <c r="I15">
-        <v>396331</v>
+        <v>396.331</v>
       </c>
       <c r="J15">
-        <v>402736</v>
+        <v>402.736</v>
       </c>
       <c r="K15">
-        <v>408854</v>
+        <v>408.854</v>
       </c>
       <c r="L15">
-        <v>410634</v>
+        <v>410.634</v>
       </c>
       <c r="M15">
-        <v>411504</v>
+        <v>411.504</v>
       </c>
       <c r="N15">
-        <v>412591</v>
+        <v>412.591</v>
       </c>
       <c r="O15">
-        <v>414029</v>
+        <v>414.029</v>
       </c>
       <c r="P15">
-        <v>415710</v>
+        <v>415.71</v>
       </c>
       <c r="Q15">
-        <v>417510</v>
+        <v>417.51</v>
       </c>
       <c r="R15">
-        <v>418293</v>
+        <v>418.293</v>
       </c>
       <c r="S15">
-        <v>418305</v>
+        <v>418.305</v>
       </c>
       <c r="T15">
-        <v>417695</v>
+        <v>417.695</v>
       </c>
       <c r="U15">
-        <v>417065</v>
+        <v>417.065</v>
       </c>
       <c r="V15">
-        <v>416598</v>
+        <v>416.598</v>
       </c>
       <c r="W15">
-        <v>416059</v>
+        <v>416.059</v>
       </c>
       <c r="X15">
-        <v>415069</v>
+        <v>415.069</v>
       </c>
       <c r="Y15">
-        <v>413414</v>
+        <v>413.414</v>
       </c>
       <c r="Z15">
-        <v>411070</v>
+        <v>411.07</v>
       </c>
       <c r="AA15">
-        <v>407982</v>
+        <v>407.982</v>
       </c>
     </row>
     <row r="16" spans="1:27">
@@ -1846,70 +1846,70 @@
         <v>66</v>
       </c>
       <c r="F16">
-        <v>75560</v>
+        <v>75.56</v>
       </c>
       <c r="G16">
-        <v>94514</v>
+        <v>94.514</v>
       </c>
       <c r="H16">
-        <v>106565</v>
+        <v>106.565</v>
       </c>
       <c r="I16">
-        <v>109869</v>
+        <v>109.869</v>
       </c>
       <c r="J16">
-        <v>115306</v>
+        <v>115.306</v>
       </c>
       <c r="K16">
-        <v>119291</v>
+        <v>119.291</v>
       </c>
       <c r="L16">
-        <v>121192</v>
+        <v>121.192</v>
       </c>
       <c r="M16">
-        <v>123331</v>
+        <v>123.331</v>
       </c>
       <c r="N16">
-        <v>124895</v>
+        <v>124.895</v>
       </c>
       <c r="O16">
-        <v>126023</v>
+        <v>126.023</v>
       </c>
       <c r="P16">
-        <v>126722</v>
+        <v>126.722</v>
       </c>
       <c r="Q16">
-        <v>126858</v>
+        <v>126.858</v>
       </c>
       <c r="R16">
-        <v>126435</v>
+        <v>126.435</v>
       </c>
       <c r="S16">
-        <v>125434</v>
+        <v>125.434</v>
       </c>
       <c r="T16">
-        <v>123993</v>
+        <v>123.993</v>
       </c>
       <c r="U16">
-        <v>122254</v>
+        <v>122.254</v>
       </c>
       <c r="V16">
-        <v>120290</v>
+        <v>120.29</v>
       </c>
       <c r="W16">
-        <v>118143</v>
+        <v>118.143</v>
       </c>
       <c r="X16">
-        <v>115856</v>
+        <v>115.856</v>
       </c>
       <c r="Y16">
-        <v>113482</v>
+        <v>113.482</v>
       </c>
       <c r="Z16">
-        <v>111055</v>
+        <v>111.055</v>
       </c>
       <c r="AA16">
-        <v>108574</v>
+        <v>108.574</v>
       </c>
     </row>
     <row r="17" spans="1:27">
@@ -1929,70 +1929,70 @@
         <v>66</v>
       </c>
       <c r="F17">
-        <v>10587</v>
+        <v>10.587</v>
       </c>
       <c r="G17">
-        <v>11237</v>
+        <v>11.237</v>
       </c>
       <c r="H17">
-        <v>12384</v>
+        <v>12.384</v>
       </c>
       <c r="I17">
-        <v>13066</v>
+        <v>13.066</v>
       </c>
       <c r="J17">
-        <v>13841</v>
+        <v>13.841</v>
       </c>
       <c r="K17">
-        <v>14504</v>
+        <v>14.504</v>
       </c>
       <c r="L17">
-        <v>14820</v>
+        <v>14.82</v>
       </c>
       <c r="M17">
-        <v>15119</v>
+        <v>15.119</v>
       </c>
       <c r="N17">
-        <v>15401</v>
+        <v>15.401</v>
       </c>
       <c r="O17">
-        <v>15680</v>
+        <v>15.68</v>
       </c>
       <c r="P17">
-        <v>15970</v>
+        <v>15.97</v>
       </c>
       <c r="Q17">
-        <v>16286</v>
+        <v>16.286</v>
       </c>
       <c r="R17">
-        <v>16562</v>
+        <v>16.562</v>
       </c>
       <c r="S17">
-        <v>16799</v>
+        <v>16.799</v>
       </c>
       <c r="T17">
-        <v>16992</v>
+        <v>16.992</v>
       </c>
       <c r="U17">
-        <v>17165</v>
+        <v>17.165</v>
       </c>
       <c r="V17">
-        <v>17326</v>
+        <v>17.326</v>
       </c>
       <c r="W17">
-        <v>17458</v>
+        <v>17.458</v>
       </c>
       <c r="X17">
-        <v>17542</v>
+        <v>17.542</v>
       </c>
       <c r="Y17">
-        <v>17574</v>
+        <v>17.574</v>
       </c>
       <c r="Z17">
-        <v>17566</v>
+        <v>17.566</v>
       </c>
       <c r="AA17">
-        <v>17526</v>
+        <v>17.526</v>
       </c>
     </row>
     <row r="18" spans="1:27">
@@ -2012,70 +2012,70 @@
         <v>66</v>
       </c>
       <c r="F18">
-        <v>623524</v>
+        <v>623.524</v>
       </c>
       <c r="G18">
-        <v>870452</v>
+        <v>870.452</v>
       </c>
       <c r="H18">
-        <v>1154640</v>
+        <v>1154.64</v>
       </c>
       <c r="I18">
-        <v>1240610</v>
+        <v>1240.61</v>
       </c>
       <c r="J18">
-        <v>1322870</v>
+        <v>1322.87</v>
       </c>
       <c r="K18">
-        <v>1407560</v>
+        <v>1407.56</v>
       </c>
       <c r="L18">
-        <v>1452180</v>
+        <v>1452.18</v>
       </c>
       <c r="M18">
-        <v>1508690</v>
+        <v>1508.69</v>
       </c>
       <c r="N18">
-        <v>1555240</v>
+        <v>1555.24</v>
       </c>
       <c r="O18">
-        <v>1591030</v>
+        <v>1591.03</v>
       </c>
       <c r="P18">
-        <v>1615150</v>
+        <v>1615.15</v>
       </c>
       <c r="Q18">
-        <v>1627870</v>
+        <v>1627.87</v>
       </c>
       <c r="R18">
-        <v>1632600</v>
+        <v>1632.6</v>
       </c>
       <c r="S18">
-        <v>1630090</v>
+        <v>1630.09</v>
       </c>
       <c r="T18">
-        <v>1619620</v>
+        <v>1619.62</v>
       </c>
       <c r="U18">
-        <v>1602070</v>
+        <v>1602.07</v>
       </c>
       <c r="V18">
-        <v>1577300</v>
+        <v>1577.3</v>
       </c>
       <c r="W18">
-        <v>1546630</v>
+        <v>1546.63</v>
       </c>
       <c r="X18">
-        <v>1511960</v>
+        <v>1511.96</v>
       </c>
       <c r="Y18">
-        <v>1475070</v>
+        <v>1475.07</v>
       </c>
       <c r="Z18">
-        <v>1436800</v>
+        <v>1436.8</v>
       </c>
       <c r="AA18">
-        <v>1398060</v>
+        <v>1398.06</v>
       </c>
     </row>
     <row r="19" spans="1:27">
@@ -2095,70 +2095,70 @@
         <v>66</v>
       </c>
       <c r="F19">
-        <v>131213</v>
+        <v>131.213</v>
       </c>
       <c r="G19">
-        <v>182160</v>
+        <v>182.16</v>
       </c>
       <c r="H19">
-        <v>228805</v>
+        <v>228.805</v>
       </c>
       <c r="I19">
-        <v>244016</v>
+        <v>244.016</v>
       </c>
       <c r="J19">
-        <v>259092</v>
+        <v>259.092</v>
       </c>
       <c r="K19">
-        <v>273753</v>
+        <v>273.753</v>
       </c>
       <c r="L19">
-        <v>281674</v>
+        <v>281.674</v>
       </c>
       <c r="M19">
-        <v>291598</v>
+        <v>291.598</v>
       </c>
       <c r="N19">
-        <v>299683</v>
+        <v>299.683</v>
       </c>
       <c r="O19">
-        <v>305698</v>
+        <v>305.698</v>
       </c>
       <c r="P19">
-        <v>309677</v>
+        <v>309.677</v>
       </c>
       <c r="Q19">
-        <v>311687</v>
+        <v>311.687</v>
       </c>
       <c r="R19">
-        <v>312298</v>
+        <v>312.298</v>
       </c>
       <c r="S19">
-        <v>311593</v>
+        <v>311.593</v>
       </c>
       <c r="T19">
-        <v>309739</v>
+        <v>309.739</v>
       </c>
       <c r="U19">
-        <v>306900</v>
+        <v>306.9</v>
       </c>
       <c r="V19">
-        <v>303234</v>
+        <v>303.234</v>
       </c>
       <c r="W19">
-        <v>298700</v>
+        <v>298.7</v>
       </c>
       <c r="X19">
-        <v>293422</v>
+        <v>293.422</v>
       </c>
       <c r="Y19">
-        <v>287519</v>
+        <v>287.519</v>
       </c>
       <c r="Z19">
-        <v>281099</v>
+        <v>281.099</v>
       </c>
       <c r="AA19">
-        <v>274310</v>
+        <v>274.31</v>
       </c>
     </row>
     <row r="20" spans="1:27">
@@ -2178,70 +2178,70 @@
         <v>66</v>
       </c>
       <c r="F20">
-        <v>112412</v>
+        <v>112.412</v>
       </c>
       <c r="G20">
-        <v>123686</v>
+        <v>123.686</v>
       </c>
       <c r="H20">
-        <v>127798</v>
+        <v>127.798</v>
       </c>
       <c r="I20">
-        <v>128105</v>
+        <v>128.105</v>
       </c>
       <c r="J20">
-        <v>127251</v>
+        <v>127.251</v>
       </c>
       <c r="K20">
-        <v>124613</v>
+        <v>124.613</v>
       </c>
       <c r="L20">
-        <v>122163</v>
+        <v>122.163</v>
       </c>
       <c r="M20">
-        <v>119046</v>
+        <v>119.046</v>
       </c>
       <c r="N20">
-        <v>115757</v>
+        <v>115.757</v>
       </c>
       <c r="O20">
-        <v>112381</v>
+        <v>112.381</v>
       </c>
       <c r="P20">
-        <v>108986</v>
+        <v>108.986</v>
       </c>
       <c r="Q20">
-        <v>105713</v>
+        <v>105.713</v>
       </c>
       <c r="R20">
-        <v>102592</v>
+        <v>102.592</v>
       </c>
       <c r="S20">
-        <v>99481</v>
+        <v>99.48099999999999</v>
       </c>
       <c r="T20">
-        <v>96196</v>
+        <v>96.196</v>
       </c>
       <c r="U20">
-        <v>92719</v>
+        <v>92.71899999999999</v>
       </c>
       <c r="V20">
-        <v>89209</v>
+        <v>89.209</v>
       </c>
       <c r="W20">
-        <v>85930</v>
+        <v>85.93000000000001</v>
       </c>
       <c r="X20">
-        <v>82962</v>
+        <v>82.962</v>
       </c>
       <c r="Y20">
-        <v>80209</v>
+        <v>80.209</v>
       </c>
       <c r="Z20">
-        <v>77538</v>
+        <v>77.538</v>
       </c>
       <c r="AA20">
-        <v>74851</v>
+        <v>74.851</v>
       </c>
     </row>
     <row r="21" spans="1:27">
@@ -2261,70 +2261,70 @@
         <v>66</v>
       </c>
       <c r="F21">
-        <v>58692</v>
+        <v>58.692</v>
       </c>
       <c r="G21">
-        <v>81720</v>
+        <v>81.72</v>
       </c>
       <c r="H21">
-        <v>105442</v>
+        <v>105.442</v>
       </c>
       <c r="I21">
-        <v>112532</v>
+        <v>112.532</v>
       </c>
       <c r="J21">
-        <v>120150</v>
+        <v>120.15</v>
       </c>
       <c r="K21">
-        <v>126705</v>
+        <v>126.705</v>
       </c>
       <c r="L21">
-        <v>130549</v>
+        <v>130.549</v>
       </c>
       <c r="M21">
-        <v>135763</v>
+        <v>135.763</v>
       </c>
       <c r="N21">
-        <v>140375</v>
+        <v>140.375</v>
       </c>
       <c r="O21">
-        <v>144253</v>
+        <v>144.253</v>
       </c>
       <c r="P21">
-        <v>147313</v>
+        <v>147.313</v>
       </c>
       <c r="Q21">
-        <v>149577</v>
+        <v>149.577</v>
       </c>
       <c r="R21">
-        <v>151213</v>
+        <v>151.213</v>
       </c>
       <c r="S21">
-        <v>152237</v>
+        <v>152.237</v>
       </c>
       <c r="T21">
-        <v>152739</v>
+        <v>152.739</v>
       </c>
       <c r="U21">
-        <v>152757</v>
+        <v>152.757</v>
       </c>
       <c r="V21">
-        <v>152317</v>
+        <v>152.317</v>
       </c>
       <c r="W21">
-        <v>151500</v>
+        <v>151.5</v>
       </c>
       <c r="X21">
-        <v>150391</v>
+        <v>150.391</v>
       </c>
       <c r="Y21">
-        <v>149048</v>
+        <v>149.048</v>
       </c>
       <c r="Z21">
-        <v>147567</v>
+        <v>147.567</v>
       </c>
       <c r="AA21">
-        <v>145892</v>
+        <v>145.892</v>
       </c>
     </row>
     <row r="22" spans="1:27">
@@ -2344,70 +2344,70 @@
         <v>66</v>
       </c>
       <c r="F22">
-        <v>79862</v>
+        <v>79.86199999999999</v>
       </c>
       <c r="G22">
-        <v>135582</v>
+        <v>135.582</v>
       </c>
       <c r="H22">
-        <v>194542</v>
+        <v>194.542</v>
       </c>
       <c r="I22">
-        <v>223614</v>
+        <v>223.614</v>
       </c>
       <c r="J22">
-        <v>249200</v>
+        <v>249.2</v>
       </c>
       <c r="K22">
-        <v>274775</v>
+        <v>274.775</v>
       </c>
       <c r="L22">
-        <v>291874</v>
+        <v>291.874</v>
       </c>
       <c r="M22">
-        <v>312900</v>
+        <v>312.9</v>
       </c>
       <c r="N22">
-        <v>332850</v>
+        <v>332.85</v>
       </c>
       <c r="O22">
-        <v>351568</v>
+        <v>351.568</v>
       </c>
       <c r="P22">
-        <v>368684</v>
+        <v>368.684</v>
       </c>
       <c r="Q22">
-        <v>383644</v>
+        <v>383.644</v>
       </c>
       <c r="R22">
-        <v>396282</v>
+        <v>396.282</v>
       </c>
       <c r="S22">
-        <v>406366</v>
+        <v>406.366</v>
       </c>
       <c r="T22">
-        <v>413733</v>
+        <v>413.733</v>
       </c>
       <c r="U22">
-        <v>418612</v>
+        <v>418.612</v>
       </c>
       <c r="V22">
-        <v>421392</v>
+        <v>421.392</v>
       </c>
       <c r="W22">
-        <v>422509</v>
+        <v>422.509</v>
       </c>
       <c r="X22">
-        <v>422396</v>
+        <v>422.396</v>
       </c>
       <c r="Y22">
-        <v>421369</v>
+        <v>421.369</v>
       </c>
       <c r="Z22">
-        <v>419452</v>
+        <v>419.452</v>
       </c>
       <c r="AA22">
-        <v>416522</v>
+        <v>416.522</v>
       </c>
     </row>
     <row r="23" spans="1:27">
@@ -2427,70 +2427,70 @@
         <v>66</v>
       </c>
       <c r="F23">
-        <v>68127</v>
+        <v>68.127</v>
       </c>
       <c r="G23">
-        <v>115414</v>
+        <v>115.414</v>
       </c>
       <c r="H23">
-        <v>174372</v>
+        <v>174.372</v>
       </c>
       <c r="I23">
-        <v>194454</v>
+        <v>194.454</v>
       </c>
       <c r="J23">
-        <v>210969</v>
+        <v>210.969</v>
       </c>
       <c r="K23">
-        <v>231402</v>
+        <v>231.402</v>
       </c>
       <c r="L23">
-        <v>250417</v>
+        <v>250.417</v>
       </c>
       <c r="M23">
-        <v>275485</v>
+        <v>275.485</v>
       </c>
       <c r="N23">
-        <v>300884</v>
+        <v>300.884</v>
       </c>
       <c r="O23">
-        <v>325815</v>
+        <v>325.815</v>
       </c>
       <c r="P23">
-        <v>349828</v>
+        <v>349.828</v>
       </c>
       <c r="Q23">
-        <v>373012</v>
+        <v>373.012</v>
       </c>
       <c r="R23">
-        <v>394733</v>
+        <v>394.733</v>
       </c>
       <c r="S23">
-        <v>414935</v>
+        <v>414.935</v>
       </c>
       <c r="T23">
-        <v>432883</v>
+        <v>432.883</v>
       </c>
       <c r="U23">
-        <v>448387</v>
+        <v>448.387</v>
       </c>
       <c r="V23">
-        <v>461249</v>
+        <v>461.249</v>
       </c>
       <c r="W23">
-        <v>471456</v>
+        <v>471.456</v>
       </c>
       <c r="X23">
-        <v>479585</v>
+        <v>479.585</v>
       </c>
       <c r="Y23">
-        <v>486094</v>
+        <v>486.094</v>
       </c>
       <c r="Z23">
-        <v>491096</v>
+        <v>491.096</v>
       </c>
       <c r="AA23">
-        <v>494804</v>
+        <v>494.804</v>
       </c>
     </row>
     <row r="24" spans="1:27">
@@ -2510,70 +2510,70 @@
         <v>66</v>
       </c>
       <c r="F24">
-        <v>133842</v>
+        <v>133.842</v>
       </c>
       <c r="G24">
-        <v>148006</v>
+        <v>148.006</v>
       </c>
       <c r="H24">
-        <v>143800</v>
+        <v>143.8</v>
       </c>
       <c r="I24">
-        <v>143243</v>
+        <v>143.243</v>
       </c>
       <c r="J24">
-        <v>144668</v>
+        <v>144.668</v>
       </c>
       <c r="K24">
-        <v>145103</v>
+        <v>145.103</v>
       </c>
       <c r="L24">
-        <v>144791</v>
+        <v>144.791</v>
       </c>
       <c r="M24">
-        <v>142828</v>
+        <v>142.828</v>
       </c>
       <c r="N24">
-        <v>141003</v>
+        <v>141.003</v>
       </c>
       <c r="O24">
-        <v>139631</v>
+        <v>139.631</v>
       </c>
       <c r="P24">
-        <v>138777</v>
+        <v>138.777</v>
       </c>
       <c r="Q24">
-        <v>138203</v>
+        <v>138.203</v>
       </c>
       <c r="R24">
-        <v>137419</v>
+        <v>137.419</v>
       </c>
       <c r="S24">
-        <v>136396</v>
+        <v>136.396</v>
       </c>
       <c r="T24">
-        <v>135082</v>
+        <v>135.082</v>
       </c>
       <c r="U24">
-        <v>133644</v>
+        <v>133.644</v>
       </c>
       <c r="V24">
-        <v>132204</v>
+        <v>132.204</v>
       </c>
       <c r="W24">
-        <v>130793</v>
+        <v>130.793</v>
       </c>
       <c r="X24">
-        <v>129417</v>
+        <v>129.417</v>
       </c>
       <c r="Y24">
-        <v>128031</v>
+        <v>128.031</v>
       </c>
       <c r="Z24">
-        <v>126538</v>
+        <v>126.538</v>
       </c>
       <c r="AA24">
-        <v>124773</v>
+        <v>124.773</v>
       </c>
     </row>
     <row r="25" spans="1:27">
@@ -2593,70 +2593,70 @@
         <v>66</v>
       </c>
       <c r="F25">
-        <v>25778</v>
+        <v>25.778</v>
       </c>
       <c r="G25">
-        <v>39878</v>
+        <v>39.878</v>
       </c>
       <c r="H25">
-        <v>49017</v>
+        <v>49.017</v>
       </c>
       <c r="I25">
-        <v>51785</v>
+        <v>51.785</v>
       </c>
       <c r="J25">
-        <v>55877</v>
+        <v>55.877</v>
       </c>
       <c r="K25">
-        <v>59392</v>
+        <v>59.392</v>
       </c>
       <c r="L25">
-        <v>61298</v>
+        <v>61.298</v>
       </c>
       <c r="M25">
-        <v>63764</v>
+        <v>63.764</v>
       </c>
       <c r="N25">
-        <v>65756</v>
+        <v>65.756</v>
       </c>
       <c r="O25">
-        <v>67295</v>
+        <v>67.295</v>
       </c>
       <c r="P25">
-        <v>68384</v>
+        <v>68.384</v>
       </c>
       <c r="Q25">
-        <v>68949</v>
+        <v>68.949</v>
       </c>
       <c r="R25">
-        <v>69100</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="S25">
-        <v>68882</v>
+        <v>68.88200000000001</v>
       </c>
       <c r="T25">
-        <v>68358</v>
+        <v>68.358</v>
       </c>
       <c r="U25">
-        <v>67546</v>
+        <v>67.54600000000001</v>
       </c>
       <c r="V25">
-        <v>66500</v>
+        <v>66.5</v>
       </c>
       <c r="W25">
-        <v>65238</v>
+        <v>65.238</v>
       </c>
       <c r="X25">
-        <v>63870</v>
+        <v>63.87</v>
       </c>
       <c r="Y25">
-        <v>62414</v>
+        <v>62.414</v>
       </c>
       <c r="Z25">
-        <v>60874</v>
+        <v>60.874</v>
       </c>
       <c r="AA25">
-        <v>59263</v>
+        <v>59.263</v>
       </c>
     </row>
     <row r="26" spans="1:27">
@@ -2676,70 +2676,70 @@
         <v>66</v>
       </c>
       <c r="F26">
-        <v>14368</v>
+        <v>14.368</v>
       </c>
       <c r="G26">
-        <v>21024</v>
+        <v>21.024</v>
       </c>
       <c r="H26">
-        <v>28146</v>
+        <v>28.146</v>
       </c>
       <c r="I26">
-        <v>30237</v>
+        <v>30.237</v>
       </c>
       <c r="J26">
-        <v>32117</v>
+        <v>32.117</v>
       </c>
       <c r="K26">
-        <v>29915</v>
+        <v>29.915</v>
       </c>
       <c r="L26">
-        <v>30883</v>
+        <v>30.883</v>
       </c>
       <c r="M26">
-        <v>32176</v>
+        <v>32.176</v>
       </c>
       <c r="N26">
-        <v>33358</v>
+        <v>33.358</v>
       </c>
       <c r="O26">
-        <v>34335</v>
+        <v>34.335</v>
       </c>
       <c r="P26">
-        <v>35092</v>
+        <v>35.092</v>
       </c>
       <c r="Q26">
-        <v>35657</v>
+        <v>35.657</v>
       </c>
       <c r="R26">
-        <v>36096</v>
+        <v>36.096</v>
       </c>
       <c r="S26">
-        <v>36437</v>
+        <v>36.437</v>
       </c>
       <c r="T26">
-        <v>36669</v>
+        <v>36.669</v>
       </c>
       <c r="U26">
-        <v>36799</v>
+        <v>36.799</v>
       </c>
       <c r="V26">
-        <v>36837</v>
+        <v>36.837</v>
       </c>
       <c r="W26">
-        <v>36791</v>
+        <v>36.791</v>
       </c>
       <c r="X26">
-        <v>36672</v>
+        <v>36.672</v>
       </c>
       <c r="Y26">
-        <v>36467</v>
+        <v>36.467</v>
       </c>
       <c r="Z26">
-        <v>36154</v>
+        <v>36.154</v>
       </c>
       <c r="AA26">
-        <v>35732</v>
+        <v>35.732</v>
       </c>
     </row>
     <row r="27" spans="1:27">
@@ -2759,70 +2759,70 @@
         <v>66</v>
       </c>
       <c r="F27">
-        <v>43901</v>
+        <v>43.901</v>
       </c>
       <c r="G27">
-        <v>60174</v>
+        <v>60.174</v>
       </c>
       <c r="H27">
-        <v>76265</v>
+        <v>76.265</v>
       </c>
       <c r="I27">
-        <v>80568</v>
+        <v>80.568</v>
       </c>
       <c r="J27">
-        <v>85449</v>
+        <v>85.449</v>
       </c>
       <c r="K27">
-        <v>93216</v>
+        <v>93.21599999999999</v>
       </c>
       <c r="L27">
-        <v>96383</v>
+        <v>96.383</v>
       </c>
       <c r="M27">
-        <v>100364</v>
+        <v>100.364</v>
       </c>
       <c r="N27">
-        <v>103774</v>
+        <v>103.774</v>
       </c>
       <c r="O27">
-        <v>106510</v>
+        <v>106.51</v>
       </c>
       <c r="P27">
-        <v>108630</v>
+        <v>108.63</v>
       </c>
       <c r="Q27">
-        <v>110157</v>
+        <v>110.157</v>
       </c>
       <c r="R27">
-        <v>111101</v>
+        <v>111.101</v>
       </c>
       <c r="S27">
-        <v>111493</v>
+        <v>111.493</v>
       </c>
       <c r="T27">
-        <v>111412</v>
+        <v>111.412</v>
       </c>
       <c r="U27">
-        <v>110905</v>
+        <v>110.905</v>
       </c>
       <c r="V27">
-        <v>109998</v>
+        <v>109.998</v>
       </c>
       <c r="W27">
-        <v>108712</v>
+        <v>108.712</v>
       </c>
       <c r="X27">
-        <v>107122</v>
+        <v>107.122</v>
       </c>
       <c r="Y27">
-        <v>105308</v>
+        <v>105.308</v>
       </c>
       <c r="Z27">
-        <v>103343</v>
+        <v>103.343</v>
       </c>
       <c r="AA27">
-        <v>101300</v>
+        <v>101.3</v>
       </c>
     </row>
     <row r="28" spans="1:27">
@@ -2842,70 +2842,70 @@
         <v>66</v>
       </c>
       <c r="F28">
-        <v>114942</v>
+        <v>114.942</v>
       </c>
       <c r="G28">
-        <v>155446</v>
+        <v>155.446</v>
       </c>
       <c r="H28">
-        <v>212253</v>
+        <v>212.253</v>
       </c>
       <c r="I28">
-        <v>225478</v>
+        <v>225.478</v>
       </c>
       <c r="J28">
-        <v>241709</v>
+        <v>241.709</v>
       </c>
       <c r="K28">
-        <v>262563</v>
+        <v>262.563</v>
       </c>
       <c r="L28">
-        <v>276432</v>
+        <v>276.432</v>
       </c>
       <c r="M28">
-        <v>292514</v>
+        <v>292.514</v>
       </c>
       <c r="N28">
-        <v>306644</v>
+        <v>306.644</v>
       </c>
       <c r="O28">
-        <v>318867</v>
+        <v>318.867</v>
       </c>
       <c r="P28">
-        <v>329242</v>
+        <v>329.242</v>
       </c>
       <c r="Q28">
-        <v>337852</v>
+        <v>337.852</v>
       </c>
       <c r="R28">
-        <v>344738</v>
+        <v>344.738</v>
       </c>
       <c r="S28">
-        <v>349742</v>
+        <v>349.742</v>
       </c>
       <c r="T28">
-        <v>353011</v>
+        <v>353.011</v>
       </c>
       <c r="U28">
-        <v>354526</v>
+        <v>354.526</v>
       </c>
       <c r="V28">
-        <v>354414</v>
+        <v>354.414</v>
       </c>
       <c r="W28">
-        <v>352723</v>
+        <v>352.723</v>
       </c>
       <c r="X28">
-        <v>349561</v>
+        <v>349.561</v>
       </c>
       <c r="Y28">
-        <v>345333</v>
+        <v>345.333</v>
       </c>
       <c r="Z28">
-        <v>340346</v>
+        <v>340.346</v>
       </c>
       <c r="AA28">
-        <v>334952</v>
+        <v>334.952</v>
       </c>
     </row>
     <row r="29" spans="1:27">
@@ -2925,70 +2925,70 @@
         <v>66</v>
       </c>
       <c r="F29">
-        <v>35931</v>
+        <v>35.931</v>
       </c>
       <c r="G29">
-        <v>44120</v>
+        <v>44.12</v>
       </c>
       <c r="H29">
-        <v>47890</v>
+        <v>47.89</v>
       </c>
       <c r="I29">
-        <v>48813</v>
+        <v>48.813</v>
       </c>
       <c r="J29">
-        <v>50994</v>
+        <v>50.994</v>
       </c>
       <c r="K29">
-        <v>51830</v>
+        <v>51.83</v>
       </c>
       <c r="L29">
-        <v>51544</v>
+        <v>51.544</v>
       </c>
       <c r="M29">
-        <v>51024</v>
+        <v>51.024</v>
       </c>
       <c r="N29">
-        <v>50296</v>
+        <v>50.296</v>
       </c>
       <c r="O29">
-        <v>49268</v>
+        <v>49.268</v>
       </c>
       <c r="P29">
-        <v>47962</v>
+        <v>47.962</v>
       </c>
       <c r="Q29">
-        <v>46502</v>
+        <v>46.502</v>
       </c>
       <c r="R29">
-        <v>44655</v>
+        <v>44.655</v>
       </c>
       <c r="S29">
-        <v>42510</v>
+        <v>42.51</v>
       </c>
       <c r="T29">
-        <v>40305</v>
+        <v>40.305</v>
       </c>
       <c r="U29">
-        <v>38185</v>
+        <v>38.185</v>
       </c>
       <c r="V29">
-        <v>36179</v>
+        <v>36.179</v>
       </c>
       <c r="W29">
-        <v>34280</v>
+        <v>34.28</v>
       </c>
       <c r="X29">
-        <v>32496</v>
+        <v>32.496</v>
       </c>
       <c r="Y29">
-        <v>30774</v>
+        <v>30.774</v>
       </c>
       <c r="Z29">
-        <v>29094</v>
+        <v>29.094</v>
       </c>
       <c r="AA29">
-        <v>27531</v>
+        <v>27.531</v>
       </c>
     </row>
     <row r="30" spans="1:27">
@@ -3008,70 +3008,70 @@
         <v>66</v>
       </c>
       <c r="F30">
-        <v>206339</v>
+        <v>206.339</v>
       </c>
       <c r="G30">
-        <v>285832</v>
+        <v>285.832</v>
       </c>
       <c r="H30">
-        <v>367521</v>
+        <v>367.521</v>
       </c>
       <c r="I30">
-        <v>391477</v>
+        <v>391.477</v>
       </c>
       <c r="J30">
-        <v>415139</v>
+        <v>415.139</v>
       </c>
       <c r="K30">
-        <v>441867</v>
+        <v>441.867</v>
       </c>
       <c r="L30">
-        <v>457865</v>
+        <v>457.865</v>
       </c>
       <c r="M30">
-        <v>475348</v>
+        <v>475.348</v>
       </c>
       <c r="N30">
-        <v>489662</v>
+        <v>489.662</v>
       </c>
       <c r="O30">
-        <v>500899</v>
+        <v>500.899</v>
       </c>
       <c r="P30">
-        <v>509310</v>
+        <v>509.31</v>
       </c>
       <c r="Q30">
-        <v>515076</v>
+        <v>515.076</v>
       </c>
       <c r="R30">
-        <v>518208</v>
+        <v>518.208</v>
       </c>
       <c r="S30">
-        <v>518721</v>
+        <v>518.721</v>
       </c>
       <c r="T30">
-        <v>517076</v>
+        <v>517.076</v>
       </c>
       <c r="U30">
-        <v>513698</v>
+        <v>513.698</v>
       </c>
       <c r="V30">
-        <v>508698</v>
+        <v>508.698</v>
       </c>
       <c r="W30">
-        <v>502372</v>
+        <v>502.372</v>
       </c>
       <c r="X30">
-        <v>494746</v>
+        <v>494.746</v>
       </c>
       <c r="Y30">
-        <v>486142</v>
+        <v>486.142</v>
       </c>
       <c r="Z30">
-        <v>476885</v>
+        <v>476.885</v>
       </c>
       <c r="AA30">
-        <v>467257</v>
+        <v>467.257</v>
       </c>
     </row>
     <row r="31" spans="1:27">
@@ -3091,70 +3091,70 @@
         <v>66</v>
       </c>
       <c r="F31">
-        <v>16552</v>
+        <v>16.552</v>
       </c>
       <c r="G31">
-        <v>20586</v>
+        <v>20.586</v>
       </c>
       <c r="H31">
-        <v>22796</v>
+        <v>22.796</v>
       </c>
       <c r="I31">
-        <v>23083</v>
+        <v>23.083</v>
       </c>
       <c r="J31">
-        <v>23512</v>
+        <v>23.512</v>
       </c>
       <c r="K31">
-        <v>23860</v>
+        <v>23.86</v>
       </c>
       <c r="L31">
-        <v>23607</v>
+        <v>23.607</v>
       </c>
       <c r="M31">
-        <v>23197</v>
+        <v>23.197</v>
       </c>
       <c r="N31">
-        <v>22659</v>
+        <v>22.659</v>
       </c>
       <c r="O31">
-        <v>21953</v>
+        <v>21.953</v>
       </c>
       <c r="P31">
-        <v>21117</v>
+        <v>21.117</v>
       </c>
       <c r="Q31">
-        <v>20222</v>
+        <v>20.222</v>
       </c>
       <c r="R31">
-        <v>19244</v>
+        <v>19.244</v>
       </c>
       <c r="S31">
-        <v>18244</v>
+        <v>18.244</v>
       </c>
       <c r="T31">
-        <v>17274</v>
+        <v>17.274</v>
       </c>
       <c r="U31">
-        <v>16332</v>
+        <v>16.332</v>
       </c>
       <c r="V31">
-        <v>15431</v>
+        <v>15.431</v>
       </c>
       <c r="W31">
-        <v>14604</v>
+        <v>14.604</v>
       </c>
       <c r="X31">
-        <v>13868</v>
+        <v>13.868</v>
       </c>
       <c r="Y31">
-        <v>13219</v>
+        <v>13.219</v>
       </c>
       <c r="Z31">
-        <v>12652</v>
+        <v>12.652</v>
       </c>
       <c r="AA31">
-        <v>12153</v>
+        <v>12.153</v>
       </c>
     </row>
     <row r="32" spans="1:27">
@@ -3174,70 +3174,70 @@
         <v>66</v>
       </c>
       <c r="F32">
-        <v>214328</v>
+        <v>214.328</v>
       </c>
       <c r="G32">
-        <v>251728</v>
+        <v>251.728</v>
       </c>
       <c r="H32">
-        <v>300755</v>
+        <v>300.755</v>
       </c>
       <c r="I32">
-        <v>315007</v>
+        <v>315.007</v>
       </c>
       <c r="J32">
-        <v>328208</v>
+        <v>328.208</v>
       </c>
       <c r="K32">
-        <v>340354</v>
+        <v>340.354</v>
       </c>
       <c r="L32">
-        <v>345517</v>
+        <v>345.517</v>
       </c>
       <c r="M32">
-        <v>353058</v>
+        <v>353.058</v>
       </c>
       <c r="N32">
-        <v>360456</v>
+        <v>360.456</v>
       </c>
       <c r="O32">
-        <v>367421</v>
+        <v>367.421</v>
       </c>
       <c r="P32">
-        <v>373815</v>
+        <v>373.815</v>
       </c>
       <c r="Q32">
-        <v>379824</v>
+        <v>379.824</v>
       </c>
       <c r="R32">
-        <v>384968</v>
+        <v>384.968</v>
       </c>
       <c r="S32">
-        <v>389941</v>
+        <v>389.941</v>
       </c>
       <c r="T32">
-        <v>394779</v>
+        <v>394.779</v>
       </c>
       <c r="U32">
-        <v>399435</v>
+        <v>399.435</v>
       </c>
       <c r="V32">
-        <v>403542</v>
+        <v>403.542</v>
       </c>
       <c r="W32">
-        <v>406575</v>
+        <v>406.575</v>
       </c>
       <c r="X32">
-        <v>408306</v>
+        <v>408.306</v>
       </c>
       <c r="Y32">
-        <v>408854</v>
+        <v>408.854</v>
       </c>
       <c r="Z32">
-        <v>408567</v>
+        <v>408.567</v>
       </c>
       <c r="AA32">
-        <v>407605</v>
+        <v>407.605</v>
       </c>
     </row>
     <row r="33" spans="1:27">
@@ -3257,70 +3257,70 @@
         <v>66</v>
       </c>
       <c r="F33">
-        <v>48892</v>
+        <v>48.892</v>
       </c>
       <c r="G33">
-        <v>51590</v>
+        <v>51.59</v>
       </c>
       <c r="H33">
-        <v>46913</v>
+        <v>46.913</v>
       </c>
       <c r="I33">
-        <v>45683</v>
+        <v>45.683</v>
       </c>
       <c r="J33">
-        <v>44983</v>
+        <v>44.983</v>
       </c>
       <c r="K33">
-        <v>43531</v>
+        <v>43.531</v>
       </c>
       <c r="L33">
-        <v>37226</v>
+        <v>37.226</v>
       </c>
       <c r="M33">
-        <v>37785</v>
+        <v>37.785</v>
       </c>
       <c r="N33">
-        <v>37779</v>
+        <v>37.779</v>
       </c>
       <c r="O33">
-        <v>37333</v>
+        <v>37.333</v>
       </c>
       <c r="P33">
-        <v>36601</v>
+        <v>36.601</v>
       </c>
       <c r="Q33">
-        <v>35770</v>
+        <v>35.77</v>
       </c>
       <c r="R33">
-        <v>34888</v>
+        <v>34.888</v>
       </c>
       <c r="S33">
-        <v>34019</v>
+        <v>34.019</v>
       </c>
       <c r="T33">
-        <v>33146</v>
+        <v>33.146</v>
       </c>
       <c r="U33">
-        <v>32289</v>
+        <v>32.289</v>
       </c>
       <c r="V33">
-        <v>31466</v>
+        <v>31.466</v>
       </c>
       <c r="W33">
-        <v>30686</v>
+        <v>30.686</v>
       </c>
       <c r="X33">
-        <v>29944</v>
+        <v>29.944</v>
       </c>
       <c r="Y33">
-        <v>29238</v>
+        <v>29.238</v>
       </c>
       <c r="Z33">
-        <v>28545</v>
+        <v>28.545</v>
       </c>
       <c r="AA33">
-        <v>27824</v>
+        <v>27.824</v>
       </c>
     </row>
     <row r="34" spans="1:27">
@@ -3340,70 +3340,70 @@
         <v>66</v>
       </c>
       <c r="F34">
-        <v>4069439</v>
+        <v>4069.439</v>
       </c>
       <c r="G34">
-        <v>5316171</v>
+        <v>5316.171</v>
       </c>
       <c r="H34">
-        <v>6558176</v>
+        <v>6558.176</v>
       </c>
       <c r="I34">
-        <v>6985595</v>
+        <v>6985.595</v>
       </c>
       <c r="J34">
-        <v>7426599</v>
+        <v>7426.599</v>
       </c>
       <c r="K34">
-        <v>7909299</v>
+        <v>7909.298999999999</v>
       </c>
       <c r="L34">
-        <v>8188939</v>
+        <v>8188.939</v>
       </c>
       <c r="M34">
-        <v>8537044</v>
+        <v>8537.044</v>
       </c>
       <c r="N34">
-        <v>8860535</v>
+        <v>8860.535</v>
       </c>
       <c r="O34">
-        <v>9157149</v>
+        <v>9157.148999999999</v>
       </c>
       <c r="P34">
-        <v>9420723</v>
+        <v>9420.723</v>
       </c>
       <c r="Q34">
-        <v>9646217</v>
+        <v>9646.217000000001</v>
       </c>
       <c r="R34">
-        <v>9829334</v>
+        <v>9829.333999999999</v>
       </c>
       <c r="S34">
-        <v>9972905</v>
+        <v>9972.905000000001</v>
       </c>
       <c r="T34">
-        <v>10078003</v>
+        <v>10078.003</v>
       </c>
       <c r="U34">
-        <v>10149932</v>
+        <v>10149.932</v>
       </c>
       <c r="V34">
-        <v>10189047</v>
+        <v>10189.047</v>
       </c>
       <c r="W34">
-        <v>10194578</v>
+        <v>10194.578</v>
       </c>
       <c r="X34">
-        <v>10169374</v>
+        <v>10169.374</v>
       </c>
       <c r="Y34">
-        <v>10118982</v>
+        <v>10118.982</v>
       </c>
       <c r="Z34">
-        <v>10046177</v>
+        <v>10046.177</v>
       </c>
       <c r="AA34">
-        <v>9951879</v>
+        <v>9951.878999999999</v>
       </c>
     </row>
     <row r="35" spans="1:27">

</xml_diff>